<commit_message>
feat: exclude security diagrams from global SVG color overrides and update week 7b data files
</commit_message>
<xml_diff>
--- a/public/data/week-7b_post_wayground.xlsx
+++ b/public/data/week-7b_post_wayground.xlsx
@@ -585,7 +585,7 @@
     <row r="3" ht="97.5" customHeight="1" s="17">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>คำสั่งในข้อใดเป็นการอนุญาตเฉพาะเครื่องไอพี 192.168.1.150 เข้าถึงพอร์ตฐานข้อมูล 3306 (TCP) ได้ถูกต้องที่สุด?</t>
+          <t>หากต้องการดูบันทึก Log UFW แบบอัปเดตสดๆ ตลอดเวลาในขณะที่เพื่อนกำลังสแกนพอร์ตเรา ควรใช้คำสั่งใด?</t>
         </is>
       </c>
       <c r="B3" s="10" t="inlineStr">
@@ -595,27 +595,27 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw allow 3306/tcp to 192.168.1.150</t>
+          <t>less /var/log/ufw.log</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw allow from 192.168.1.150 to any port 3306 proto tcp</t>
+          <t>cat /var/log/ufw.log</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw permit from 192.168.1.150 port 3306</t>
+          <t>sudo watch ufw.log</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw whitelist 192.168.1.150 on port 3306</t>
+          <t>sudo tail -f /var/log/ufw.log</t>
         </is>
       </c>
       <c r="G3" s="10" t="n"/>
       <c r="H3" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I3" s="10" t="n">
         <v>30</v>
@@ -626,7 +626,7 @@
     <row r="4" ht="12.75" customHeight="1" s="17">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>เมื่อใช้คำสั่ง sudo ufw status แล้วได้ข้อความ Status: inactive หมายความว่าอย่างไร?</t>
+          <t>คำสั่งใดใช้เพื่อเปิดใช้งานระบบ UFW Firewall ให้ทำงาน?</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -636,22 +636,22 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>ระบบ UFW กำลังค้นหาการ์ดเชื่อมต่อเครือข่ายใหม่</t>
+          <t>sudo ufw start</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>UFW Firewall ทำงานปกติแต่ไม่พบบันทึกการเชื่อมต่อใหม่</t>
+          <t>sudo ufw run</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>UFW Firewall ถูกปิดใช้งานอยู่และไม่มีผลบังคับใช้ใดๆ กับเครือข่าย</t>
+          <t>sudo ufw enable</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>ระบบปิดพอร์ตทุกพอร์ตยกเว้นพอร์ต 22 เพื่อความปลอดภัย</t>
+          <t>sudo ufw service-start</t>
         </is>
       </c>
       <c r="G4" s="10" t="n"/>
@@ -659,14 +659,14 @@
         <v>3</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="J4" s="12" t="n"/>
     </row>
     <row r="5" ht="12.75" customHeight="1" s="17">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t>เหตุใดการลบกฎไฟร์วอลล์ด้วยลำดับตัวเลข (เช่น sudo ufw delete 3) จึงเป็นที่นิยมและปลอดภัยกว่าการลบด้วยคำสั่งกฎเต็ม?</t>
+          <t>UFW ย่อมาจากคำเต็มว่าอะไร?</t>
         </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
@@ -676,22 +676,22 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>เพราะช่วยลดความเสี่ยงในการสะกดไวยากรณ์กฎผิดพลาดและลบได้รวดเร็ว</t>
+          <t>Uncomplicated Firewall</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>เพื่อหลีกเลี่ยงไม่ให้ CPU ทำงานหนักเกินไปจากการค้นหาคำสั่ง</t>
+          <t>User Friendly Website</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>เพื่อป้องกันไม่ให้แอปพลิเคชัน Nginx ตรวจเจอการเปลี่ยนแปลงระบบ</t>
+          <t>Unified Flow Window</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>เป็นกฎบังคับทางกฎหมายคอมพิวเตอร์ของการจัดการไฟร์วอลล์</t>
+          <t>Universal File Wrapper</t>
         </is>
       </c>
       <c r="G5" s="10" t="n"/>
@@ -706,7 +706,7 @@
     <row r="6" ht="12.75" customHeight="1" s="17">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>คำสั่งใดใช้ในการปิดการทำงานของ UFW Firewall บนตู้ Ubuntu เซิร์ฟเวอร์อย่างถาวร?</t>
+          <t>ใน UFW Log ไฟล์ /var/log/ufw.log ค่าตัวย่อ DPT และ SRC ย่อมาจากอะไรตามลำดับ?</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
@@ -716,37 +716,37 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw stop</t>
+          <t>Database Port และ Security Router Connection</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw disable</t>
+          <t>Data Packet Type และ Server Rule Code</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw shutdown</t>
+          <t>Direction Policy และ Source Port</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw deactivate</t>
+          <t>Destination Port (พอร์ตปลายทาง) และ Source IP (ไอพีผู้ส่งต้นทาง)</t>
         </is>
       </c>
       <c r="G6" s="14" t="n"/>
       <c r="H6" s="11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="J6" s="10" t="n"/>
     </row>
     <row r="7" ht="12.75" customHeight="1" s="17">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>หากเราสั่ง telnet [IP ปลายทาง] 80 แล้วขึ้นสถานะ Connection timed out ยาวนานโดยไม่มีการตอบกลับ หมายความว่าอะไร?</t>
+          <t>คำสั่งในข้อใดเป็นการอนุญาตเฉพาะเครื่องไอพี 192.168.1.150 เข้าถึงพอร์ตฐานข้อมูล 3306 (TCP) ได้ถูกต้องที่สุด?</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
@@ -756,27 +756,27 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>พอร์ต 80 ของเซิร์ฟเวอร์ปิดการใช้งานและปฏิเสธสัญญาณทันที (REJECT)</t>
+          <t>sudo ufw permit from 192.168.1.150 port 3306</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>มีไฟร์วอลล์ของเซิร์ฟเวอร์เป้าหมายสกัดกั้นสัญญาณไว้ (DROP)</t>
+          <t>sudo ufw allow 3306/tcp to 192.168.1.150</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>เซิร์ฟเวอร์เป้าหมายกำลังรัน MariaDB ที่พอร์ต 80 แทน Nginx</t>
+          <t>sudo ufw allow from 192.168.1.150 to any port 3306 proto tcp</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
-          <t>สายแลนเครือข่ายของเซิร์ฟเวอร์เป้าหมายถูกถอดออกทันที</t>
+          <t>sudo ufw whitelist 192.168.1.150 on port 3306</t>
         </is>
       </c>
       <c r="G7" s="10" t="n"/>
       <c r="H7" s="11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I7" s="10" t="n">
         <v>30</v>
@@ -786,7 +786,7 @@
     <row r="8" ht="12.75" customHeight="1" s="17">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>ใน UFW Log ไฟล์ /var/log/ufw.log ค่าตัวย่อ DPT และ SRC ย่อมาจากอะไรตามลำดับ?</t>
+          <t>กฎ UFW เริ่มต้น (Default Policy) หลังจากติดตั้งมักถูกกำหนดไว้อย่างไรเพื่อความปลอดภัยสูงสุด?</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -796,37 +796,37 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Data Packet Type และ Server Rule Code</t>
+          <t>เปิดบริการทุกพอร์ตโดยไม่มีการตรวจสอบใดๆ</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Database Port และ Security Router Connection</t>
+          <t>บล็อกสัญญาณเข้าทั้งหมด และอนุญาตสัญญาณออกทั้งหมด</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
         <is>
-          <t>Destination Port (พอร์ตปลายทาง) และ Source IP (ไอพีผู้ส่งต้นทาง)</t>
+          <t>บล็อกทั้งสัญญาณเข้าและออกทั้งหมด</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Direction Policy และ Source Port</t>
+          <t>อนุญาตสัญญาณเข้าทั้งหมด และบล็อกสัญญาณออกทั้งหมด</t>
         </is>
       </c>
       <c r="G8" s="14" t="n"/>
       <c r="H8" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="J8" s="10" t="n"/>
     </row>
     <row r="9" ht="12.75" customHeight="1" s="17">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>หากต้องการจำลองสแกนพอร์ตเป้าหมายอย่างรวดเร็ว เฉพาะ 100 พอร์ตยอดนิยม ด้วย Nmap แบบ SYN Stealth Scan ควรพิมพ์คำสั่งอย่างไร?</t>
+          <t>ถ้าต้องการเปิดพอร์ต 80 (HTTP) เฉพาะโปรโตคอล TCP ควรพิมพ์คำสั่งอย่างไร?</t>
         </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
@@ -836,37 +836,37 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>nmap -sS -F [IP]</t>
+          <t>sudo ufw open port 80</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>nmap -sV -p 1-65535 [IP]</t>
+          <t>sudo ufw permit tcp 80</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>nmap --fast-scan [IP]</t>
+          <t>sudo ufw allow 80/tcp</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
-          <t>nmap localhost -F</t>
+          <t>sudo ufw add rule 80 tcp</t>
         </is>
       </c>
       <c r="G9" s="14" t="n"/>
       <c r="H9" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="J9" s="10" t="n"/>
     </row>
     <row r="10" ht="12.75" customHeight="1" s="17">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>การบล็อก IP เดี่ยว (deny from 192.168.10.15) เทียบกับการบล็อก Subnet /24 (deny from 192.168.10.0/24) มีผลลัพธ์ต่างกันอย่างไร?</t>
+          <t>หากต้องการบล็อกทุกการเชื่อมต่อจากไอพี 192.168.1.50 ไม่ให้เข้าเซิร์ฟเวอร์ของเรา ควรเขียนคำสั่งอย่างไร?</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
@@ -876,22 +876,22 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>การบล็อกแบบ Subnet จะสแกนหาเฉพาะเครื่องคอมพิวเตอร์ที่เป็นเซิร์ฟเวอร์หลัก</t>
+          <t>sudo ufw reject to 192.168.1.50</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>การบล็อกแบบ Subnet จะปิดกั้นไอพีทั้งหมดตั้งแต่ .0 ถึง .255 ในวงแลนนั้น</t>
+          <t>sudo ufw deny from 192.168.1.50</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>การบล็อกแบบเดี่ยวมีความปลอดภัยและทำงานได้เร็วกว่าการบล็อกแบบ Subnet 10 เท่า</t>
+          <t>sudo ufw drop 192.168.1.50</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>ไม่มีความแตกต่างกันในแง่ของจำนวนไอพีที่ถูกปิดกั้น</t>
+          <t>sudo ufw block 192.168.1.50</t>
         </is>
       </c>
       <c r="G10" s="14" t="n"/>
@@ -916,22 +916,22 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
+          <t>ufw block-abuse 22</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>ufw limit 22/tcp</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>ufw ssh-secure</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
           <t>ufw deny 22/tcp</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>ufw limit 22/tcp</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>ufw block-abuse 22</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>ufw ssh-secure</t>
         </is>
       </c>
       <c r="G11" s="14" t="n"/>
@@ -946,7 +946,7 @@
     <row r="12" ht="12.75" customHeight="1" s="17">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>กฎข้อใดของ UFW ในคลาสเรียนที่จะทำให้เพื่อนร่วมห้อง (ไอพี 192.168.1.180) ไม่สามารถสแกนพอร์ตหรือเชื่อมต่อใดๆ กับเครื่องคุณได้เลย?</t>
+          <t>ไฟล์ใดในเซิร์ฟเวอร์ Ubuntu ที่ทำหน้าที่บันทึกประวัติเหตุการณ์สกัดกั้นข้อมูลของ UFW (Firewall Log)?</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
@@ -956,30 +956,30 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>sudo ufw deny to 192.168.1.180</t>
+          <t>/var/log/ufw.log</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>sudo ufw deny from 192.168.1.180 to any</t>
+          <t>/var/log/syslog/ufw.log</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw block ip 192.168.1.180</t>
+          <t>/etc/ufw/rules.log</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>sudo ufw reject port all to 192.168.1.180</t>
+          <t>/var/log/nginx/access.log</t>
         </is>
       </c>
       <c r="G12" s="14" t="n"/>
       <c r="H12" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="J12" s="10" t="n"/>
     </row>

</xml_diff>